<commit_message>
Lock ATMCS 13 travel at £2,150 for University approval.
Sync the 21 Oct Stockholm planner through the JeS cost pack, capability note, timeline, and V&A dissemination wording before institutional review.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/08_current/grant/live/Costs/ATMCS_13_travel_budget.xlsx
+++ b/08_current/grant/live/Costs/ATMCS_13_travel_budget.xlsx
@@ -37,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,20 +45,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -425,30 +417,30 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
     <col width="36" customWidth="1" min="3" max="3"/>
-    <col width="6" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="42" customWidth="1" min="7" max="7"/>
-    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>ATMCS 13 travel budget — APP98322 / IPA 799 (16 Oct 2026) — PL ONLY</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ATMCS 13 travel budget — APP98322 / IPA 799 (21 Oct 2026) — PL ONLY</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Meeting: ATMCS 13, KTH Stockholm, 28 Jun–2 Jul 2027</t>
+          <t>Meeting: ATMCS 13, KTH Stockholm, conference 28 Jun–2 Jul 2027; travel window 26 Jun–3 Jul 2027</t>
         </is>
       </c>
     </row>
@@ -462,7 +454,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>FX planning: SEK 1 = GBP 0.073 (16 Oct 2026). HMRC Stockholm OSR.</t>
+          <t>Source: Travel budget planner 21 10 26 IPA 799.xlsx. FX: xe.com 21/10/26 (~SEK 1 = GBP 0.075). HMRC Stockholm OSR.</t>
         </is>
       </c>
     </row>
@@ -472,356 +464,284 @@
           <t>Code</t>
         </is>
       </c>
-      <c r="B6" s="1" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C6" s="1" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="D6" s="1" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="E6" s="1" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>Unit_GBP</t>
         </is>
       </c>
-      <c r="F6" s="1" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>Total_GBP</t>
         </is>
       </c>
-      <c r="G6" s="1" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>Basis</t>
         </is>
       </c>
-      <c r="H6" s="1" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>Audit_evidence</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>REG-PL</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>Registration</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>Conference registration, PL</t>
         </is>
       </c>
-      <c r="D7" s="2" t="n">
+      <c r="D7" t="n">
         <v>1</v>
       </c>
-      <c r="E7" s="2" t="n">
-        <v>280</v>
-      </c>
-      <c r="F7" s="2" t="n">
-        <v>280</v>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>ATMCS11 early USD300 precedent + uplift</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="E7" t="n">
+        <v>375</v>
+      </c>
+      <c r="F7" t="n">
+        <v>375</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Planner 21 Oct 2026</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
         <is>
           <t>ATMCS invoice + payment proof</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>FLT-PL</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>Flights</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>Economy return UK–ARN, PL</t>
         </is>
       </c>
-      <c r="D8" s="2" t="n">
+      <c r="D8" t="n">
         <v>1</v>
       </c>
-      <c r="E8" s="2" t="n">
-        <v>250</v>
-      </c>
-      <c r="F8" s="2" t="n">
-        <v>250</v>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>Book ≥3 months ahead</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="E8" t="n">
+        <v>170</v>
+      </c>
+      <c r="F8" t="n">
+        <v>170</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Planner 21 Oct 2026</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
         <is>
           <t>E-ticket + boarding passes</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>TRN</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Train / ground</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>UK airport rail + Arlanda–Stockholm</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" t="n">
+        <v>100</v>
+      </c>
+      <c r="F9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Planner train line</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Tickets</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>HOT-PL</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>Accommodation</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Hotel nights 27 Jun–2 Jul</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="E9" s="2" t="n">
-        <v>142</v>
-      </c>
-      <c r="F9" s="2" t="n">
-        <v>710</v>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>HMRC Stockholm room SEK 1939.50 × 0.073</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Hotel nights 26 Jun–3 Jul</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>7</v>
+      </c>
+      <c r="E10" t="n">
+        <v>146</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1022</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>HMRC room SEK 1939.50 → £146</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
         <is>
           <t>Hotel invoice named guest</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
           <t>SUB-PL</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>Subsistence</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>Food + local transit residual</t>
         </is>
       </c>
-      <c r="D10" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="E10" s="2" t="n">
-        <v>67</v>
-      </c>
-      <c r="F10" s="2" t="n">
-        <v>335</v>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>HMRC Stockholm residual SEK 917.50 × 0.073</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="D11" t="n">
+        <v>7</v>
+      </c>
+      <c r="E11" t="n">
+        <v>69</v>
+      </c>
+      <c r="F11" t="n">
+        <v>483</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>HMRC residual SEK 917.50 → £69</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
         <is>
           <t>Itinerary</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>TRN-UK</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Transfers</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>UK rail/coach to airport</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E11" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="F11" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>Actual vouchers</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>Ticket</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>TRN-SE</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Transfers</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Arlanda–Stockholm link</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E12" s="2" t="n">
-        <v>35</v>
-      </c>
-      <c r="F12" s="2" t="n">
-        <v>35</v>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>Arlanda Express / Flygbussarna</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>Ticket</t>
-        </is>
-      </c>
-    </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>CON</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>Contingency</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>FX / fare / late fee buffer</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E13" s="2" t="n">
-        <v>165</v>
-      </c>
-      <c r="F13" s="2" t="n">
-        <v>165</v>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>Only against coded overruns</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>Note on claim if used</t>
-        </is>
+      <c r="A13" t="inlineStr"/>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>TRAVEL TOTAL</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="n">
+        <v>2150</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>JeS DI Travel</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>PL only</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Staff total fEC</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>96918</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr"/>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>TRAVEL TOTAL</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" s="3" t="n">
-        <v>1800</v>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>JeS DI Travel</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>PL only</t>
-        </is>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Travel DI</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>2150</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Staff total fEC</t>
+          <t>Project total with travel</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>96918</v>
+        <v>99068</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Travel DI</t>
+          <t>Unused headroom to £100k</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>1800</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Project total with travel</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>98718</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Unused headroom to £100k</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>1282</v>
+        <v>932</v>
       </c>
     </row>
   </sheetData>

</xml_diff>